<commit_message>
feat(shared): human-readable Czech column names in population XLSX
Parser now accepts both new readable names (Věk, Pohlaví, Vzdělání,
Stav, Partner, Status, Příjem, Životní příběh) and legacy technical
names (Vek, Pohlavi, Vzdelani, etc.) for backward compatibility.

Export updated to use new readable names. Template regenerated with
20 sample persons matching expected test IDs (P001–P020).

Security fixes:
- Deduplicate optional fields via findColumnForField to prevent
  silent last-write-wins when both name variants are present
- Guard custom field export against collision with fixed column names
- Remove unused parseSuccess import and dead REQUIRED_FIELD_COLUMNS
- Add ZamestnaneckyStatus ASCII legacy alias alongside diacritic form

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/sample-population.xlsx
+++ b/templates/sample-population.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Osoby" sheetId="1" r:id="rId1"/>
-    <sheet name="Metadata" sheetId="2" r:id="rId2"/>
+    <sheet name="Nápověda" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -400,15 +400,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J21"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="6.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="5.83203125" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="32.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -417,31 +417,31 @@
         <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>Vek</v>
+        <v>Věk</v>
       </c>
       <c r="C1" t="str">
-        <v>Pohlavi</v>
+        <v>Pohlaví</v>
       </c>
       <c r="D1" t="str">
-        <v>Vzdelani</v>
+        <v>Vzdělání</v>
       </c>
       <c r="E1" t="str">
-        <v>RodinnyStav</v>
+        <v>Stav</v>
       </c>
       <c r="F1" t="str">
-        <v>MaPartnera</v>
+        <v>Partner</v>
       </c>
       <c r="G1" t="str">
-        <v>ZaměstnaneckyStatus</v>
+        <v>Status</v>
       </c>
       <c r="H1" t="str">
-        <v>PrijmoveRozpeti</v>
+        <v>Příjem</v>
       </c>
       <c r="I1" t="str">
         <v>Kraj</v>
       </c>
       <c r="J1" t="str">
-        <v>ZivotniPribeh</v>
+        <v>Životní příběh</v>
       </c>
     </row>
     <row r="2">
@@ -458,7 +458,7 @@
         <v>Vysokoškolské</v>
       </c>
       <c r="E2" t="str">
-        <v>Ženatý/Vdaná</v>
+        <v>Svobodný/á</v>
       </c>
       <c r="F2" t="str">
         <v>Ano</v>
@@ -467,13 +467,13 @@
         <v>Zaměstnaný/á</v>
       </c>
       <c r="H2" t="str">
-        <v>Střední</v>
+        <v>Spíše vyšší</v>
       </c>
       <c r="I2" t="str">
         <v>Praha</v>
       </c>
       <c r="J2" t="str">
-        <v>Vystudoval ekonomii na VŠE, pracuje jako finanční analytik v nadnárodní firmě. Žije v Praze s manželkou a dvěma dětmi. Politicky se považuje za středopravicového.</v>
+        <v>Vystudoval informatiku na ČVUT. Pracuje jako softwarový inženýr v pražském startupu. Ve volném čase rád čte a chodí na výlety do přírody.</v>
       </c>
     </row>
     <row r="3">
@@ -481,7 +481,7 @@
         <v>P002</v>
       </c>
       <c r="B3">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C3" t="str">
         <v>Žena</v>
@@ -499,13 +499,13 @@
         <v>Důchodce/kyně</v>
       </c>
       <c r="H3" t="str">
-        <v>Nízký</v>
+        <v>Střední</v>
       </c>
       <c r="I3" t="str">
-        <v>Moravskoslezský</v>
+        <v>Jihomoravský</v>
       </c>
       <c r="J3" t="str">
-        <v>Celý život pracovala jako zdravotní sestra v ostravské nemocnici. Ovdověla před třemi lety, bydlí sama v panelákovém bytě. Ráda zahradničí a sleduje seriály.</v>
+        <v>Celý život pracovala jako účetní. Po odchodu do důchodu se věnuje zahrádkaření a vnoučatům.</v>
       </c>
     </row>
     <row r="4">
@@ -513,28 +513,28 @@
         <v>P003</v>
       </c>
       <c r="B4">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="C4" t="str">
-        <v>Žena</v>
+        <v>Muž</v>
       </c>
       <c r="D4" t="str">
-        <v>S maturitou</v>
+        <v>Vyučení</v>
       </c>
       <c r="E4" t="str">
-        <v>Svobodný/á</v>
+        <v>Ženatý/Vdaná</v>
       </c>
       <c r="F4" t="str">
         <v>Ano</v>
       </c>
       <c r="G4" t="str">
-        <v>Student/ka</v>
+        <v>Zaměstnaný/á</v>
       </c>
       <c r="H4" t="str">
-        <v>Nízký</v>
+        <v>Střední</v>
       </c>
       <c r="I4" t="str">
-        <v>Jihomoravský</v>
+        <v>Moravskoslezský</v>
       </c>
       <c r="J4" t="str">
         <v/>
@@ -545,28 +545,28 @@
         <v>P004</v>
       </c>
       <c r="B5">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="C5" t="str">
-        <v>Muž</v>
+        <v>Žena</v>
       </c>
       <c r="D5" t="str">
-        <v>Vyučení</v>
+        <v>Vysokoškolské</v>
       </c>
       <c r="E5" t="str">
-        <v>Rozvedený/á</v>
+        <v>Svobodný/á</v>
       </c>
       <c r="F5" t="str">
-        <v>Ne</v>
+        <v>Ano</v>
       </c>
       <c r="G5" t="str">
         <v>Zaměstnaný/á</v>
       </c>
       <c r="H5" t="str">
-        <v>Spíše nižší</v>
+        <v>Nízký</v>
       </c>
       <c r="I5" t="str">
-        <v>Ústecký</v>
+        <v>Praha</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -577,13 +577,13 @@
         <v>P005</v>
       </c>
       <c r="B6">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="C6" t="str">
-        <v>Žena</v>
+        <v>Muž</v>
       </c>
       <c r="D6" t="str">
-        <v>Vysokoškolské</v>
+        <v>S maturitou</v>
       </c>
       <c r="E6" t="str">
         <v>Ženatý/Vdaná</v>
@@ -592,10 +592,10 @@
         <v>Ano</v>
       </c>
       <c r="G6" t="str">
-        <v>Mateřská/rodičovská dovolená</v>
+        <v>Důchodce/kyně</v>
       </c>
       <c r="H6" t="str">
-        <v>Spíše vyšší</v>
+        <v>Spíše nižší</v>
       </c>
       <c r="I6" t="str">
         <v>Středočeský</v>
@@ -609,28 +609,28 @@
         <v>P006</v>
       </c>
       <c r="B7">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C7" t="str">
-        <v>Muž</v>
+        <v>Žena</v>
       </c>
       <c r="D7" t="str">
-        <v>Vysokoškolské</v>
+        <v>Vyšší odborné</v>
       </c>
       <c r="E7" t="str">
-        <v>Ženatý/Vdaná</v>
+        <v>Rozvedený/á</v>
       </c>
       <c r="F7" t="str">
-        <v>Ano</v>
+        <v>Ne</v>
       </c>
       <c r="G7" t="str">
-        <v>Podnikatel/ka (OSVČ)</v>
+        <v>Zaměstnaný/á</v>
       </c>
       <c r="H7" t="str">
-        <v>Vysoký</v>
+        <v>Střední</v>
       </c>
       <c r="I7" t="str">
-        <v>Praha</v>
+        <v>Plzeňský</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -641,25 +641,25 @@
         <v>P007</v>
       </c>
       <c r="B8">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C8" t="str">
         <v>Muž</v>
       </c>
       <c r="D8" t="str">
-        <v>Vysokoškolské</v>
+        <v>S maturitou</v>
       </c>
       <c r="E8" t="str">
-        <v>Svobodný/á</v>
+        <v>Ženatý/Vdaná</v>
       </c>
       <c r="F8" t="str">
         <v>Ano</v>
       </c>
       <c r="G8" t="str">
-        <v>Zaměstnaný/á</v>
+        <v>Podnikatel/ka (OSVČ)</v>
       </c>
       <c r="H8" t="str">
-        <v>Střední</v>
+        <v>Vysoký</v>
       </c>
       <c r="I8" t="str">
         <v>Jihočeský</v>
@@ -673,13 +673,13 @@
         <v>P008</v>
       </c>
       <c r="B9">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="C9" t="str">
-        <v>Muž</v>
+        <v>Žena</v>
       </c>
       <c r="D9" t="str">
-        <v>Základní</v>
+        <v>Vysokoškolské</v>
       </c>
       <c r="E9" t="str">
         <v>Ženatý/Vdaná</v>
@@ -688,13 +688,13 @@
         <v>Ano</v>
       </c>
       <c r="G9" t="str">
-        <v>Důchodce/kyně</v>
+        <v>Mateřská/rodičovská dovolená</v>
       </c>
       <c r="H9" t="str">
-        <v>Nízký</v>
+        <v>Střední</v>
       </c>
       <c r="I9" t="str">
-        <v>Kraj Vysočina</v>
+        <v>Jihomoravský</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -705,13 +705,13 @@
         <v>P009</v>
       </c>
       <c r="B10">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="C10" t="str">
-        <v>Žena</v>
+        <v>Muž</v>
       </c>
       <c r="D10" t="str">
-        <v>Vyšší odborné</v>
+        <v>S maturitou</v>
       </c>
       <c r="E10" t="str">
         <v>Svobodný/á</v>
@@ -720,13 +720,13 @@
         <v>Ne</v>
       </c>
       <c r="G10" t="str">
-        <v>Zaměstnaný/á</v>
+        <v>Student/ka</v>
       </c>
       <c r="H10" t="str">
-        <v>Střední</v>
+        <v>Nízký</v>
       </c>
       <c r="I10" t="str">
-        <v>Plzeňský</v>
+        <v>Olomoucký</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -737,28 +737,28 @@
         <v>P010</v>
       </c>
       <c r="B11">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C11" t="str">
         <v>Žena</v>
       </c>
       <c r="D11" t="str">
-        <v>S maturitou</v>
+        <v>Základní</v>
       </c>
       <c r="E11" t="str">
-        <v>Ženatý/Vdaná</v>
+        <v>Rozvedený/á</v>
       </c>
       <c r="F11" t="str">
-        <v>Ano</v>
+        <v>Ne</v>
       </c>
       <c r="G11" t="str">
-        <v>Zaměstnaný/á</v>
+        <v>Nezaměstnaný/á</v>
       </c>
       <c r="H11" t="str">
-        <v>Střední</v>
+        <v>Nízký</v>
       </c>
       <c r="I11" t="str">
-        <v>Olomoucký</v>
+        <v>Ústecký</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -769,28 +769,28 @@
         <v>P011</v>
       </c>
       <c r="B12">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="C12" t="str">
         <v>Muž</v>
       </c>
       <c r="D12" t="str">
-        <v>S maturitou</v>
+        <v>Vysokoškolské</v>
       </c>
       <c r="E12" t="str">
-        <v>Svobodný/á</v>
+        <v>Ženatý/Vdaná</v>
       </c>
       <c r="F12" t="str">
-        <v>Ne</v>
+        <v>Ano</v>
       </c>
       <c r="G12" t="str">
         <v>Zaměstnaný/á</v>
       </c>
       <c r="H12" t="str">
-        <v>Spíše nižší</v>
+        <v>Spíše vyšší</v>
       </c>
       <c r="I12" t="str">
-        <v>Liberecký</v>
+        <v>Praha</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -801,7 +801,7 @@
         <v>P012</v>
       </c>
       <c r="B13">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C13" t="str">
         <v>Žena</v>
@@ -816,7 +816,7 @@
         <v>Ano</v>
       </c>
       <c r="G13" t="str">
-        <v>Zaměstnaný/á</v>
+        <v>Důchodce/kyně</v>
       </c>
       <c r="H13" t="str">
         <v>Spíše nižší</v>
@@ -833,28 +833,28 @@
         <v>P013</v>
       </c>
       <c r="B14">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="C14" t="str">
-        <v>Muž</v>
+        <v>Žena</v>
       </c>
       <c r="D14" t="str">
-        <v>Vysokoškolské</v>
+        <v>S maturitou</v>
       </c>
       <c r="E14" t="str">
-        <v>Rozvedený/á</v>
+        <v>Svobodný/á</v>
       </c>
       <c r="F14" t="str">
-        <v>Ano</v>
+        <v>Ne</v>
       </c>
       <c r="G14" t="str">
-        <v>Podnikatel/ka (OSVČ)</v>
+        <v>Zaměstnaný/á</v>
       </c>
       <c r="H14" t="str">
-        <v>Spíše vyšší</v>
+        <v>Nízký</v>
       </c>
       <c r="I14" t="str">
-        <v>Královéhradecký</v>
+        <v>Liberecký</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -865,28 +865,28 @@
         <v>P014</v>
       </c>
       <c r="B15">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="C15" t="str">
-        <v>Žena</v>
+        <v>Muž</v>
       </c>
       <c r="D15" t="str">
-        <v>S maturitou</v>
+        <v>Vyšší odborné</v>
       </c>
       <c r="E15" t="str">
-        <v>Svobodný/á</v>
+        <v>Ženatý/Vdaná</v>
       </c>
       <c r="F15" t="str">
-        <v>Ne</v>
+        <v>Ano</v>
       </c>
       <c r="G15" t="str">
-        <v>Student/ka</v>
+        <v>Zaměstnaný/á</v>
       </c>
       <c r="H15" t="str">
-        <v>Nízký</v>
+        <v>Střední</v>
       </c>
       <c r="I15" t="str">
-        <v>Pardubický</v>
+        <v>Karlovarský</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -897,28 +897,28 @@
         <v>P015</v>
       </c>
       <c r="B16">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="C16" t="str">
-        <v>Muž</v>
+        <v>Žena</v>
       </c>
       <c r="D16" t="str">
-        <v>Vyučení</v>
+        <v>Vysokoškolské</v>
       </c>
       <c r="E16" t="str">
-        <v>Ženatý/Vdaná</v>
+        <v>Svobodný/á</v>
       </c>
       <c r="F16" t="str">
         <v>Ano</v>
       </c>
       <c r="G16" t="str">
-        <v>Důchodce/kyně</v>
+        <v>Zaměstnaný/á</v>
       </c>
       <c r="H16" t="str">
         <v>Střední</v>
       </c>
       <c r="I16" t="str">
-        <v>Karlovarský</v>
+        <v>Pardubický</v>
       </c>
       <c r="J16" t="str">
         <v/>
@@ -929,28 +929,28 @@
         <v>P016</v>
       </c>
       <c r="B17">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="C17" t="str">
-        <v>Žena</v>
+        <v>Muž</v>
       </c>
       <c r="D17" t="str">
-        <v>Vysokoškolské</v>
+        <v>S maturitou</v>
       </c>
       <c r="E17" t="str">
-        <v>Svobodný/á</v>
+        <v>Ovdovělý/á</v>
       </c>
       <c r="F17" t="str">
-        <v>Ano</v>
+        <v>Ne</v>
       </c>
       <c r="G17" t="str">
-        <v>Zaměstnaný/á</v>
+        <v>Důchodce/kyně</v>
       </c>
       <c r="H17" t="str">
-        <v>Spíše vyšší</v>
+        <v>Střední</v>
       </c>
       <c r="I17" t="str">
-        <v>Praha</v>
+        <v>Královéhradecký</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -961,13 +961,13 @@
         <v>P017</v>
       </c>
       <c r="B18">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="C18" t="str">
-        <v>Muž</v>
+        <v>Žena</v>
       </c>
       <c r="D18" t="str">
-        <v>S maturitou</v>
+        <v>Základní</v>
       </c>
       <c r="E18" t="str">
         <v>Ženatý/Vdaná</v>
@@ -976,13 +976,13 @@
         <v>Ano</v>
       </c>
       <c r="G18" t="str">
-        <v>Zaměstnaný/á</v>
+        <v>Nezaměstnaný/á</v>
       </c>
       <c r="H18" t="str">
-        <v>Střední</v>
+        <v>Nízký</v>
       </c>
       <c r="I18" t="str">
-        <v>Jihomoravský</v>
+        <v>Moravskoslezský</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -993,16 +993,16 @@
         <v>P018</v>
       </c>
       <c r="B19">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="C19" t="str">
         <v>Muž</v>
       </c>
       <c r="D19" t="str">
-        <v>Vysokoškolské</v>
+        <v>Vyučení</v>
       </c>
       <c r="E19" t="str">
-        <v>Svobodný/á</v>
+        <v>Rozvedený/á</v>
       </c>
       <c r="F19" t="str">
         <v>Ne</v>
@@ -1011,10 +1011,10 @@
         <v>Zaměstnaný/á</v>
       </c>
       <c r="H19" t="str">
-        <v>Střední</v>
+        <v>Spíše nižší</v>
       </c>
       <c r="I19" t="str">
-        <v>Středočeský</v>
+        <v>Kraj Vysočina</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1025,31 +1025,31 @@
         <v>P019</v>
       </c>
       <c r="B20">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C20" t="str">
         <v>Žena</v>
       </c>
       <c r="D20" t="str">
-        <v>Vyučení</v>
+        <v>S maturitou</v>
       </c>
       <c r="E20" t="str">
-        <v>Rozvedený/á</v>
+        <v>Ženatý/Vdaná</v>
       </c>
       <c r="F20" t="str">
-        <v>Ne</v>
+        <v>Ano</v>
       </c>
       <c r="G20" t="str">
-        <v>Nezaměstnaný/á</v>
+        <v>Podnikatel/ka (OSVČ)</v>
       </c>
       <c r="H20" t="str">
-        <v>Nízký</v>
+        <v>Spíše vyšší</v>
       </c>
       <c r="I20" t="str">
-        <v>Ústecký</v>
+        <v>Jihočeský</v>
       </c>
       <c r="J20" t="str">
-        <v>Po rozvodu zůstala sama se dvěma dětmi. Přišla o práci v továrně před rokem. Aktivně hledá práci, ale na trhu v regionu není mnoho příležitostí.</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1057,28 +1057,28 @@
         <v>P020</v>
       </c>
       <c r="B21">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="C21" t="str">
-        <v>Žena</v>
+        <v>Muž</v>
       </c>
       <c r="D21" t="str">
-        <v>Základní</v>
+        <v>S maturitou</v>
       </c>
       <c r="E21" t="str">
-        <v>Ovdovělý/á</v>
+        <v>Svobodný/á</v>
       </c>
       <c r="F21" t="str">
         <v>Ne</v>
       </c>
       <c r="G21" t="str">
-        <v>Důchodce/kyně</v>
+        <v>Student/ka</v>
       </c>
       <c r="H21" t="str">
         <v>Nízký</v>
       </c>
       <c r="I21" t="str">
-        <v>Moravskoslezský</v>
+        <v>Středočeský</v>
       </c>
       <c r="J21" t="str">
         <v/>
@@ -1093,59 +1093,171 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D11"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="55.83203125" customWidth="1"/>
+    <col min="4" max="4" width="100.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Pole</v>
+        <v>Sloupec</v>
       </c>
       <c r="B1" t="str">
-        <v>Hodnota</v>
+        <v>Povinné</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Popis</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Povolené hodnoty</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Název</v>
+        <v>ID</v>
       </c>
       <c r="B2" t="str">
-        <v>Vzorová populace Respondex</v>
+        <v>Ano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Unikátní identifikátor osoby (libovolný řetězec)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>P001, R0001, OSOBA_001, ...</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Popis</v>
+        <v>Věk</v>
       </c>
       <c r="B3" t="str">
-        <v>Ukázková populace 20 osob pokrývající různé demografické skupiny české populace</v>
+        <v>Ano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Věk v celých letech, rozsah 18–100</v>
+      </c>
+      <c r="D3" t="str">
+        <v>celé číslo 18–100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Zdroj</v>
+        <v>Pohlaví</v>
       </c>
       <c r="B4" t="str">
-        <v>Ručně sestaveno pro demonstraci platformy Respondex</v>
+        <v>Ano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Pohlaví osoby</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Muž | Žena</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Datum</v>
+        <v>Vzdělání</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-03-21</v>
+        <v>Ne</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nejvyšší dosažené vzdělání</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Základní | Vyučení | S maturitou | Vyšší odborné | Vysokoškolské</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Verze</v>
+        <v>Stav</v>
       </c>
       <c r="B6" t="str">
-        <v>1.0</v>
+        <v>Ne</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Rodinný stav</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Svobodný/á | Ženatý/Vdaná | Rozvedený/á | Ovdovělý/á | Registrované partnerství</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Partner</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Má aktuálního partnera/partnerku</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Ano | Ne</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Pracovní status</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Zaměstnaný/á | Podnikatel/ka (OSVČ) | Nezaměstnaný/á | Student/ka | Důchodce/kyně | Mateřská/rodičovská dovolená | Jiné</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Příjem</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Příjmová skupina</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Nízký | Spíše nižší | Střední | Spíše vyšší | Vysoký</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Kraj</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Kraj bydliště</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Praha | Středočeský | Jihočeský | Plzeňský | Karlovarský | Ústecký | Liberecký | Královéhradecký | Pardubický | Kraj Vysočina | Jihomoravský | Olomoucký | Zlínský | Moravskoslezský</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Životní příběh</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Volný text s životním příběhem (pro Strategii C — manuální narativ)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>libovolný text</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>